<commit_message>
Creando nueva clausula de temporadas + 1er gráfico
</commit_message>
<xml_diff>
--- a/alcohol_filtrado.xlsx
+++ b/alcohol_filtrado.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F247"/>
+  <dimension ref="A1:G247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,11 @@
           <t>rango</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>temporada</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -469,6 +474,11 @@
       <c r="F2" t="n">
         <v>2.59</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -491,6 +501,11 @@
       <c r="F3" t="n">
         <v>2.57</v>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -513,6 +528,11 @@
       <c r="F4" t="n">
         <v>2.6</v>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -535,6 +555,11 @@
       <c r="F5" t="n">
         <v>2.65</v>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -557,6 +582,11 @@
       <c r="F6" t="n">
         <v>2.5</v>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -579,6 +609,11 @@
       <c r="F7" t="n">
         <v>2.79</v>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -601,6 +636,11 @@
       <c r="F8" t="n">
         <v>3.91</v>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -623,6 +663,11 @@
       <c r="F9" t="n">
         <v>3.77</v>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -645,6 +690,11 @@
       <c r="F10" t="n">
         <v>3.74</v>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -667,6 +717,11 @@
       <c r="F11" t="n">
         <v>3.42</v>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -689,6 +744,11 @@
       <c r="F12" t="n">
         <v>3.26</v>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -711,6 +771,11 @@
       <c r="F13" t="n">
         <v>3.41</v>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -733,6 +798,11 @@
       <c r="F14" t="n">
         <v>3.82</v>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -755,6 +825,11 @@
       <c r="F15" t="n">
         <v>3.98</v>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -777,6 +852,11 @@
       <c r="F16" t="n">
         <v>3.93</v>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -799,6 +879,11 @@
       <c r="F17" t="n">
         <v>3.97</v>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -821,6 +906,11 @@
       <c r="F18" t="n">
         <v>3.51</v>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -843,6 +933,11 @@
       <c r="F19" t="n">
         <v>3.49</v>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -865,6 +960,11 @@
       <c r="F20" t="n">
         <v>3.33</v>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -887,6 +987,11 @@
       <c r="F21" t="n">
         <v>3.29</v>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -909,6 +1014,11 @@
       <c r="F22" t="n">
         <v>3.38</v>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -931,6 +1041,11 @@
       <c r="F23" t="n">
         <v>3.43</v>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -953,6 +1068,11 @@
       <c r="F24" t="n">
         <v>3.66</v>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -975,6 +1095,11 @@
       <c r="F25" t="n">
         <v>3.42</v>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -997,6 +1122,11 @@
       <c r="F26" t="n">
         <v>3.2</v>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1019,6 +1149,11 @@
       <c r="F27" t="n">
         <v>3.1</v>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1041,6 +1176,11 @@
       <c r="F28" t="n">
         <v>3.21</v>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1063,6 +1203,11 @@
       <c r="F29" t="n">
         <v>3.34</v>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1085,6 +1230,11 @@
       <c r="F30" t="n">
         <v>3.3</v>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1107,6 +1257,11 @@
       <c r="F31" t="n">
         <v>3.07</v>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1129,6 +1284,11 @@
       <c r="F32" t="n">
         <v>2.91</v>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1151,6 +1311,11 @@
       <c r="F33" t="n">
         <v>2.85</v>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1173,6 +1338,11 @@
       <c r="F34" t="n">
         <v>2.64</v>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1195,6 +1365,11 @@
       <c r="F35" t="n">
         <v>2.68</v>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1217,6 +1392,11 @@
       <c r="F36" t="n">
         <v>2.77</v>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1239,6 +1419,11 @@
       <c r="F37" t="n">
         <v>2.91</v>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1261,6 +1446,11 @@
       <c r="F38" t="n">
         <v>3.59</v>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1283,6 +1473,11 @@
       <c r="F39" t="n">
         <v>3.61</v>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1305,6 +1500,11 @@
       <c r="F40" t="n">
         <v>3.55</v>
       </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1327,6 +1527,11 @@
       <c r="F41" t="n">
         <v>3.59</v>
       </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1349,6 +1554,11 @@
       <c r="F42" t="n">
         <v>3.81</v>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1371,6 +1581,11 @@
       <c r="F43" t="n">
         <v>3.62</v>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1393,6 +1608,11 @@
       <c r="F44" t="n">
         <v>3.82</v>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1415,6 +1635,11 @@
       <c r="F45" t="n">
         <v>3.59</v>
       </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1437,6 +1662,11 @@
       <c r="F46" t="n">
         <v>3.61</v>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1459,6 +1689,11 @@
       <c r="F47" t="n">
         <v>3.69</v>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1481,6 +1716,11 @@
       <c r="F48" t="n">
         <v>3.67</v>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1503,6 +1743,11 @@
       <c r="F49" t="n">
         <v>3.65</v>
       </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1525,6 +1770,11 @@
       <c r="F50" t="n">
         <v>2.89</v>
       </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1547,6 +1797,11 @@
       <c r="F51" t="n">
         <v>3.17</v>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1569,6 +1824,11 @@
       <c r="F52" t="n">
         <v>3.02</v>
       </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1591,6 +1851,11 @@
       <c r="F53" t="n">
         <v>2.9</v>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1613,6 +1878,11 @@
       <c r="F54" t="n">
         <v>2.68</v>
       </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1635,6 +1905,11 @@
       <c r="F55" t="n">
         <v>2.55</v>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1657,6 +1932,11 @@
       <c r="F56" t="n">
         <v>3.85</v>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1679,6 +1959,11 @@
       <c r="F57" t="n">
         <v>3.78</v>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1701,6 +1986,11 @@
       <c r="F58" t="n">
         <v>3.72</v>
       </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1723,6 +2013,11 @@
       <c r="F59" t="n">
         <v>3.89</v>
       </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1745,6 +2040,11 @@
       <c r="F60" t="n">
         <v>3.6</v>
       </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1767,6 +2067,11 @@
       <c r="F61" t="n">
         <v>3.77</v>
       </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1789,6 +2094,11 @@
       <c r="F62" t="n">
         <v>3.53</v>
       </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1811,6 +2121,11 @@
       <c r="F63" t="n">
         <v>3.6</v>
       </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1833,6 +2148,11 @@
       <c r="F64" t="n">
         <v>3.45</v>
       </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1855,6 +2175,11 @@
       <c r="F65" t="n">
         <v>3.32</v>
       </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1877,6 +2202,11 @@
       <c r="F66" t="n">
         <v>3.35</v>
       </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1899,6 +2229,11 @@
       <c r="F67" t="n">
         <v>3.4</v>
       </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1921,6 +2256,11 @@
       <c r="F68" t="n">
         <v>5.94</v>
       </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1943,6 +2283,11 @@
       <c r="F69" t="n">
         <v>5.44</v>
       </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1965,6 +2310,11 @@
       <c r="F70" t="n">
         <v>5.1</v>
       </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1987,6 +2337,11 @@
       <c r="F71" t="n">
         <v>4.64</v>
       </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2009,6 +2364,11 @@
       <c r="F72" t="n">
         <v>4.82</v>
       </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2031,6 +2391,11 @@
       <c r="F73" t="n">
         <v>4.72</v>
       </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2053,6 +2418,11 @@
       <c r="F74" t="n">
         <v>3.81</v>
       </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2075,6 +2445,11 @@
       <c r="F75" t="n">
         <v>3.9</v>
       </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2097,6 +2472,11 @@
       <c r="F76" t="n">
         <v>3.79</v>
       </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2119,6 +2499,11 @@
       <c r="F77" t="n">
         <v>3.86</v>
       </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2141,6 +2526,11 @@
       <c r="F78" t="n">
         <v>3.6</v>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2163,6 +2553,11 @@
       <c r="F79" t="n">
         <v>3.4</v>
       </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2185,6 +2580,11 @@
       <c r="F80" t="n">
         <v>3.59</v>
       </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2207,6 +2607,11 @@
       <c r="F81" t="n">
         <v>3.77</v>
       </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2229,6 +2634,11 @@
       <c r="F82" t="n">
         <v>3.77</v>
       </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2251,6 +2661,11 @@
       <c r="F83" t="n">
         <v>3.61</v>
       </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2273,6 +2688,11 @@
       <c r="F84" t="n">
         <v>3.64</v>
       </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2295,6 +2715,11 @@
       <c r="F85" t="n">
         <v>3.59</v>
       </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2317,6 +2742,11 @@
       <c r="F86" t="n">
         <v>3.56</v>
       </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2339,6 +2769,11 @@
       <c r="F87" t="n">
         <v>3.39</v>
       </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2361,6 +2796,11 @@
       <c r="F88" t="n">
         <v>3.37</v>
       </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2383,6 +2823,11 @@
       <c r="F89" t="n">
         <v>3.55</v>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2405,6 +2850,11 @@
       <c r="F90" t="n">
         <v>3.6</v>
       </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2427,6 +2877,11 @@
       <c r="F91" t="n">
         <v>3.47</v>
       </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2449,6 +2904,11 @@
       <c r="F92" t="n">
         <v>3.06</v>
       </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2471,6 +2931,11 @@
       <c r="F93" t="n">
         <v>3.04</v>
       </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2493,6 +2958,11 @@
       <c r="F94" t="n">
         <v>2.92</v>
       </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2515,6 +2985,11 @@
       <c r="F95" t="n">
         <v>3.04</v>
       </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2537,6 +3012,11 @@
       <c r="F96" t="n">
         <v>2.88</v>
       </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2559,6 +3039,11 @@
       <c r="F97" t="n">
         <v>2.9</v>
       </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2581,6 +3066,11 @@
       <c r="F98" t="n">
         <v>3.5</v>
       </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2603,6 +3093,11 @@
       <c r="F99" t="n">
         <v>3.67</v>
       </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2625,6 +3120,11 @@
       <c r="F100" t="n">
         <v>3.58</v>
       </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2647,6 +3147,11 @@
       <c r="F101" t="n">
         <v>3.64</v>
       </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2669,6 +3174,11 @@
       <c r="F102" t="n">
         <v>3.58</v>
       </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2691,6 +3201,11 @@
       <c r="F103" t="n">
         <v>3.41</v>
       </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2713,6 +3228,11 @@
       <c r="F104" t="n">
         <v>3.39</v>
       </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2735,6 +3255,11 @@
       <c r="F105" t="n">
         <v>3.32</v>
       </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2757,6 +3282,11 @@
       <c r="F106" t="n">
         <v>3.45</v>
       </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2779,6 +3309,11 @@
       <c r="F107" t="n">
         <v>3.29</v>
       </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2801,6 +3336,11 @@
       <c r="F108" t="n">
         <v>3.17</v>
       </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2823,6 +3363,11 @@
       <c r="F109" t="n">
         <v>3.03</v>
       </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2845,6 +3390,11 @@
       <c r="F110" t="n">
         <v>3.47</v>
       </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2867,6 +3417,11 @@
       <c r="F111" t="n">
         <v>3.61</v>
       </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2889,6 +3444,11 @@
       <c r="F112" t="n">
         <v>3.47</v>
       </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2911,6 +3471,11 @@
       <c r="F113" t="n">
         <v>3.64</v>
       </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2933,6 +3498,11 @@
       <c r="F114" t="n">
         <v>3.49</v>
       </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2955,6 +3525,11 @@
       <c r="F115" t="n">
         <v>3.47</v>
       </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2977,6 +3552,11 @@
       <c r="F116" t="n">
         <v>2.7</v>
       </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2999,6 +3579,11 @@
       <c r="F117" t="n">
         <v>2.68</v>
       </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3021,6 +3606,11 @@
       <c r="F118" t="n">
         <v>2.77</v>
       </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3043,6 +3633,11 @@
       <c r="F119" t="n">
         <v>2.96</v>
       </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3065,6 +3660,11 @@
       <c r="F120" t="n">
         <v>3.04</v>
       </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3087,6 +3687,11 @@
       <c r="F121" t="n">
         <v>3.03</v>
       </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3109,6 +3714,11 @@
       <c r="F122" t="n">
         <v>5.09</v>
       </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3131,6 +3741,11 @@
       <c r="F123" t="n">
         <v>5.1</v>
       </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3153,6 +3768,11 @@
       <c r="F124" t="n">
         <v>5.2</v>
       </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3175,6 +3795,11 @@
       <c r="F125" t="n">
         <v>4.88</v>
       </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3197,6 +3822,11 @@
       <c r="F126" t="n">
         <v>4.85</v>
       </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3219,6 +3849,11 @@
       <c r="F127" t="n">
         <v>4.67</v>
       </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3241,6 +3876,11 @@
       <c r="F128" t="n">
         <v>4.02</v>
       </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3263,6 +3903,11 @@
       <c r="F129" t="n">
         <v>3.79</v>
       </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -3285,6 +3930,11 @@
       <c r="F130" t="n">
         <v>3.64</v>
       </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -3307,6 +3957,11 @@
       <c r="F131" t="n">
         <v>3.59</v>
       </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -3329,6 +3984,11 @@
       <c r="F132" t="n">
         <v>3.65</v>
       </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -3351,6 +4011,11 @@
       <c r="F133" t="n">
         <v>3.51</v>
       </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -3373,6 +4038,11 @@
       <c r="F134" t="n">
         <v>3.6</v>
       </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -3395,6 +4065,11 @@
       <c r="F135" t="n">
         <v>3.6</v>
       </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -3417,6 +4092,11 @@
       <c r="F136" t="n">
         <v>3.7</v>
       </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -3439,6 +4119,11 @@
       <c r="F137" t="n">
         <v>3.58</v>
       </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -3461,6 +4146,11 @@
       <c r="F138" t="n">
         <v>3.61</v>
       </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -3483,6 +4173,11 @@
       <c r="F139" t="n">
         <v>3.53</v>
       </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -3505,6 +4200,11 @@
       <c r="F140" t="n">
         <v>3.25</v>
       </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -3527,6 +4227,11 @@
       <c r="F141" t="n">
         <v>3.21</v>
       </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -3549,6 +4254,11 @@
       <c r="F142" t="n">
         <v>3.34</v>
       </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3571,6 +4281,11 @@
       <c r="F143" t="n">
         <v>3.11</v>
       </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3593,6 +4308,11 @@
       <c r="F144" t="n">
         <v>2.93</v>
       </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3615,6 +4335,11 @@
       <c r="F145" t="n">
         <v>2.79</v>
       </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3637,6 +4362,11 @@
       <c r="F146" t="n">
         <v>4.26</v>
       </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3659,6 +4389,11 @@
       <c r="F147" t="n">
         <v>4.09</v>
       </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -3681,6 +4416,11 @@
       <c r="F148" t="n">
         <v>4.15</v>
       </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -3703,6 +4443,11 @@
       <c r="F149" t="n">
         <v>4.16</v>
       </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -3725,6 +4470,11 @@
       <c r="F150" t="n">
         <v>4.15</v>
       </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -3747,6 +4497,11 @@
       <c r="F151" t="n">
         <v>4.19</v>
       </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -3769,6 +4524,11 @@
       <c r="F152" t="n">
         <v>3.45</v>
       </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -3791,6 +4551,11 @@
       <c r="F153" t="n">
         <v>3.55</v>
       </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -3813,6 +4578,11 @@
       <c r="F154" t="n">
         <v>3.43</v>
       </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -3835,6 +4605,11 @@
       <c r="F155" t="n">
         <v>3.48</v>
       </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -3857,6 +4632,11 @@
       <c r="F156" t="n">
         <v>3.24</v>
       </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -3879,6 +4659,11 @@
       <c r="F157" t="n">
         <v>3.18</v>
       </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -3901,6 +4686,11 @@
       <c r="F158" t="n">
         <v>3.14</v>
       </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -3923,6 +4713,11 @@
       <c r="F159" t="n">
         <v>2.98</v>
       </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -3945,6 +4740,11 @@
       <c r="F160" t="n">
         <v>3.24</v>
       </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -3967,6 +4767,11 @@
       <c r="F161" t="n">
         <v>3.13</v>
       </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3989,6 +4794,11 @@
       <c r="F162" t="n">
         <v>2.99</v>
       </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -4011,6 +4821,11 @@
       <c r="F163" t="n">
         <v>3.04</v>
       </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -4033,6 +4848,11 @@
       <c r="F164" t="n">
         <v>2.77</v>
       </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -4055,6 +4875,11 @@
       <c r="F165" t="n">
         <v>2.7</v>
       </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -4077,6 +4902,11 @@
       <c r="F166" t="n">
         <v>2.52</v>
       </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -4099,6 +4929,11 @@
       <c r="F167" t="n">
         <v>2.56</v>
       </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -4121,6 +4956,11 @@
       <c r="F168" t="n">
         <v>2.62</v>
       </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -4143,6 +4983,11 @@
       <c r="F169" t="n">
         <v>2.67</v>
       </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -4165,6 +5010,11 @@
       <c r="F170" t="n">
         <v>2.73</v>
       </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -4187,6 +5037,11 @@
       <c r="F171" t="n">
         <v>2.7</v>
       </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -4209,6 +5064,11 @@
       <c r="F172" t="n">
         <v>2.85</v>
       </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -4231,6 +5091,11 @@
       <c r="F173" t="n">
         <v>2.71</v>
       </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -4253,6 +5118,11 @@
       <c r="F174" t="n">
         <v>2.76</v>
       </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -4275,6 +5145,11 @@
       <c r="F175" t="n">
         <v>2.83</v>
       </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -4297,6 +5172,11 @@
       <c r="F176" t="n">
         <v>3.64</v>
       </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -4319,6 +5199,11 @@
       <c r="F177" t="n">
         <v>3.83</v>
       </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -4341,6 +5226,11 @@
       <c r="F178" t="n">
         <v>3.86</v>
       </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -4363,6 +5253,11 @@
       <c r="F179" t="n">
         <v>3.86</v>
       </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -4385,6 +5280,11 @@
       <c r="F180" t="n">
         <v>3.71</v>
       </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -4407,6 +5307,11 @@
       <c r="F181" t="n">
         <v>3.72</v>
       </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -4429,6 +5334,11 @@
       <c r="F182" t="n">
         <v>3.47</v>
       </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -4451,6 +5361,11 @@
       <c r="F183" t="n">
         <v>3.64</v>
       </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -4473,6 +5388,11 @@
       <c r="F184" t="n">
         <v>3.58</v>
       </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -4495,6 +5415,11 @@
       <c r="F185" t="n">
         <v>3.29</v>
       </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -4517,6 +5442,11 @@
       <c r="F186" t="n">
         <v>3.42</v>
       </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -4539,6 +5469,11 @@
       <c r="F187" t="n">
         <v>3.52</v>
       </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -4561,6 +5496,11 @@
       <c r="F188" t="n">
         <v>5.18</v>
       </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -4583,6 +5523,11 @@
       <c r="F189" t="n">
         <v>5.36</v>
       </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -4605,6 +5550,11 @@
       <c r="F190" t="n">
         <v>5.09</v>
       </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -4627,6 +5577,11 @@
       <c r="F191" t="n">
         <v>5.34</v>
       </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -4649,6 +5604,11 @@
       <c r="F192" t="n">
         <v>5.24</v>
       </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -4671,6 +5631,11 @@
       <c r="F193" t="n">
         <v>5.23</v>
       </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -4693,6 +5658,11 @@
       <c r="F194" t="n">
         <v>4.04</v>
       </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -4715,6 +5685,11 @@
       <c r="F195" t="n">
         <v>3.95</v>
       </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -4737,6 +5712,11 @@
       <c r="F196" t="n">
         <v>3.93</v>
       </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -4759,6 +5739,11 @@
       <c r="F197" t="n">
         <v>3.93</v>
       </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -4781,6 +5766,11 @@
       <c r="F198" t="n">
         <v>3.96</v>
       </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -4803,6 +5793,11 @@
       <c r="F199" t="n">
         <v>3.97</v>
       </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -4825,6 +5820,11 @@
       <c r="F200" t="n">
         <v>3.38</v>
       </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -4847,6 +5847,11 @@
       <c r="F201" t="n">
         <v>3.29</v>
       </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -4869,6 +5874,11 @@
       <c r="F202" t="n">
         <v>3.22</v>
       </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -4891,6 +5901,11 @@
       <c r="F203" t="n">
         <v>3.24</v>
       </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -4913,6 +5928,11 @@
       <c r="F204" t="n">
         <v>3.37</v>
       </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -4935,6 +5955,11 @@
       <c r="F205" t="n">
         <v>3.36</v>
       </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -4957,6 +5982,11 @@
       <c r="F206" t="n">
         <v>3.4</v>
       </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -4979,6 +6009,11 @@
       <c r="F207" t="n">
         <v>3.59</v>
       </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -5001,6 +6036,11 @@
       <c r="F208" t="n">
         <v>3.42</v>
       </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -5023,6 +6063,11 @@
       <c r="F209" t="n">
         <v>3.43</v>
       </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -5045,6 +6090,11 @@
       <c r="F210" t="n">
         <v>3.45</v>
       </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -5067,6 +6117,11 @@
       <c r="F211" t="n">
         <v>3.53</v>
       </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -5089,6 +6144,11 @@
       <c r="F212" t="n">
         <v>3.6</v>
       </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -5111,6 +6171,11 @@
       <c r="F213" t="n">
         <v>3.48</v>
       </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -5133,6 +6198,11 @@
       <c r="F214" t="n">
         <v>3.62</v>
       </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -5155,6 +6225,11 @@
       <c r="F215" t="n">
         <v>3.5</v>
       </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -5177,6 +6252,11 @@
       <c r="F216" t="n">
         <v>3.67</v>
       </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -5199,6 +6279,11 @@
       <c r="F217" t="n">
         <v>3.51</v>
       </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -5221,6 +6306,11 @@
       <c r="F218" t="n">
         <v>3.47</v>
       </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -5243,6 +6333,11 @@
       <c r="F219" t="n">
         <v>3.51</v>
       </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -5265,6 +6360,11 @@
       <c r="F220" t="n">
         <v>3.71</v>
       </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -5287,6 +6387,11 @@
       <c r="F221" t="n">
         <v>3.5</v>
       </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -5309,6 +6414,11 @@
       <c r="F222" t="n">
         <v>3.44</v>
       </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -5331,6 +6441,11 @@
       <c r="F223" t="n">
         <v>3.42</v>
       </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -5353,6 +6468,11 @@
       <c r="F224" t="n">
         <v>3.76</v>
       </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -5375,6 +6495,11 @@
       <c r="F225" t="n">
         <v>3.75</v>
       </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -5397,6 +6522,11 @@
       <c r="F226" t="n">
         <v>3.58</v>
       </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -5419,6 +6549,11 @@
       <c r="F227" t="n">
         <v>3.44</v>
       </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -5441,6 +6576,11 @@
       <c r="F228" t="n">
         <v>3.46</v>
       </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -5463,6 +6603,11 @@
       <c r="F229" t="n">
         <v>3.61</v>
       </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -5485,6 +6630,11 @@
       <c r="F230" t="n">
         <v>3.38</v>
       </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -5507,6 +6657,11 @@
       <c r="F231" t="n">
         <v>3.25</v>
       </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -5529,6 +6684,11 @@
       <c r="F232" t="n">
         <v>3.32</v>
       </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -5551,6 +6711,11 @@
       <c r="F233" t="n">
         <v>3.18</v>
       </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -5573,6 +6738,11 @@
       <c r="F234" t="n">
         <v>3.11</v>
       </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -5595,6 +6765,11 @@
       <c r="F235" t="n">
         <v>3.19</v>
       </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -5617,6 +6792,11 @@
       <c r="F236" t="n">
         <v>3.59</v>
       </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -5639,6 +6819,11 @@
       <c r="F237" t="n">
         <v>3.62</v>
       </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -5661,6 +6846,11 @@
       <c r="F238" t="n">
         <v>3.76</v>
       </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -5683,6 +6873,11 @@
       <c r="F239" t="n">
         <v>3.62</v>
       </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -5705,6 +6900,11 @@
       <c r="F240" t="n">
         <v>3.54</v>
       </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -5727,6 +6927,11 @@
       <c r="F241" t="n">
         <v>3.42</v>
       </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -5749,6 +6954,11 @@
       <c r="F242" t="n">
         <v>3.61</v>
       </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -5771,6 +6981,11 @@
       <c r="F243" t="n">
         <v>3.37</v>
       </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -5793,6 +7008,11 @@
       <c r="F244" t="n">
         <v>3.41</v>
       </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -5815,6 +7035,11 @@
       <c r="F245" t="n">
         <v>3.33</v>
       </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>Antes</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -5837,6 +7062,11 @@
       <c r="F246" t="n">
         <v>3.56</v>
       </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>Durante</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -5858,6 +7088,11 @@
       </c>
       <c r="F247" t="n">
         <v>3.36</v>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>Después</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>